<commit_message>
completed profile view for employees and employee data view for companies
</commit_message>
<xml_diff>
--- a/documentation/Hire Me Project Report.xlsx
+++ b/documentation/Hire Me Project Report.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="34">
   <si>
     <t>Frontend</t>
   </si>
@@ -84,9 +84,6 @@
   </si>
   <si>
     <t>LogIn api</t>
-  </si>
-  <si>
-    <t>New Manage account creation api</t>
   </si>
   <si>
     <t>Account details fetch api</t>
@@ -136,6 +133,12 @@
   </si>
   <si>
     <t>Employee list fetch api</t>
+  </si>
+  <si>
+    <t>New Manager account creation api</t>
+  </si>
+  <si>
+    <t>Employee List</t>
   </si>
 </sst>
 </file>
@@ -659,10 +662,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>80</c:v>
+                  <c:v>75</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>20</c:v>
+                  <c:v>25</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -994,10 +997,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>40</c:v>
+                  <c:v>55</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>60</c:v>
+                  <c:v>45</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2523,7 +2526,7 @@
   <sheetData>
     <row r="1" spans="4:14" ht="31.5" x14ac:dyDescent="0.5">
       <c r="E1" s="18" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F1" s="19"/>
       <c r="G1" s="19"/>
@@ -2611,10 +2614,10 @@
       <c r="H5" s="5"/>
       <c r="I5" s="5"/>
       <c r="J5" s="4" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="4:14" ht="18.75" x14ac:dyDescent="0.3">
@@ -2629,10 +2632,10 @@
       <c r="H6" s="5"/>
       <c r="I6" s="5"/>
       <c r="J6" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="4:14" ht="18.75" x14ac:dyDescent="0.3">
@@ -2644,19 +2647,25 @@
       <c r="G7" s="4"/>
       <c r="H7" s="5"/>
       <c r="I7" s="5"/>
-      <c r="J7" s="5"/>
+      <c r="J7" s="4" t="s">
+        <v>23</v>
+      </c>
       <c r="K7" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8" spans="4:14" ht="18.75" x14ac:dyDescent="0.3">
       <c r="D8" s="6"/>
       <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
+      <c r="F8" s="4" t="s">
+        <v>33</v>
+      </c>
       <c r="G8" s="5"/>
       <c r="H8" s="5"/>
       <c r="I8" s="5"/>
-      <c r="J8" s="5"/>
+      <c r="J8" s="4" t="s">
+        <v>31</v>
+      </c>
       <c r="K8" s="5"/>
     </row>
     <row r="9" spans="4:14" ht="18.75" x14ac:dyDescent="0.3">
@@ -2664,46 +2673,38 @@
         <v>16</v>
       </c>
       <c r="E9" s="5"/>
-      <c r="F9" s="7" t="s">
-        <v>14</v>
-      </c>
       <c r="G9" s="5"/>
       <c r="H9" s="5"/>
       <c r="I9" s="5"/>
-      <c r="J9" s="7" t="s">
+      <c r="J9" s="4" t="s">
         <v>24</v>
       </c>
       <c r="K9" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="4:14" ht="18.75" x14ac:dyDescent="0.3">
       <c r="D10" s="21"/>
       <c r="E10" s="5"/>
-      <c r="F10" s="7" t="s">
-        <v>15</v>
-      </c>
       <c r="G10" s="5"/>
       <c r="H10" s="5"/>
       <c r="I10" s="5"/>
-      <c r="J10" s="7" t="s">
-        <v>32</v>
-      </c>
       <c r="K10" s="5"/>
     </row>
-    <row r="11" spans="4:14" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="J11" s="7" t="s">
-        <v>25</v>
-      </c>
-    </row>
     <row r="12" spans="4:14" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="F12" s="7" t="s">
+        <v>14</v>
+      </c>
       <c r="J12" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13" spans="4:14" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="F13" s="7" t="s">
+        <v>15</v>
+      </c>
       <c r="J13" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" spans="4:14" ht="21" x14ac:dyDescent="0.25">
@@ -2711,7 +2712,7 @@
     </row>
     <row r="18" spans="5:10" ht="26.25" x14ac:dyDescent="0.4">
       <c r="E18" s="23" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F18" s="23"/>
       <c r="G18" s="23"/>
@@ -2749,18 +2750,18 @@
     </row>
     <row r="21" spans="5:10" ht="21" x14ac:dyDescent="0.25">
       <c r="E21" s="16">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="F21" s="17">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="G21" s="10"/>
       <c r="H21" s="10"/>
       <c r="I21" s="16">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="J21" s="17">
-        <v>60</v>
+        <v>45</v>
       </c>
     </row>
     <row r="22" spans="5:10" ht="21" x14ac:dyDescent="0.35">

</xml_diff>